<commit_message>
Add Microsoft Dynamics 365 column to ERP comparison workbook
Added Dynamics 365 as the 9th product across all 54 matrix rows with
accurate Y/P/N ratings. Updated cover TOC, Where-NEXA-Wins narratives,
and the honest-caveat note to mention Dynamics. Merge refs and slice
indices updated to reflect the wider column count. Rebuilt xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NEXA-vs-ERP-Comparison.xlsx
+++ b/NEXA-vs-ERP-Comparison.xlsx
@@ -340,7 +340,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generated 2026-06-15</t>
+          <t xml:space="preserve">Generated 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -372,7 +372,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">54 capabilities scored for NEXA vs SAP S/4HANA, Tally, Tally Prime, Zoho Books, Odoo, QuickBooks, NetSuite</t>
+          <t xml:space="preserve">54 capabilities scored for NEXA vs SAP S/4HANA, Tally, Tally Prime, Zoho Books, Odoo, QuickBooks, NetSuite, and Microsoft Dynamics 365</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">NEXA is an integrated, India-statutory-first finance suite (a client-side SPA). The comparison below is about functional design, compliance depth and UX — areas where NEXA matches or beats far heavier products — not about backend scale or infrastructure, where tier-1 ERPs (SAP, NetSuite) remain the enterprise systems of record.</t>
+          <t xml:space="preserve">NEXA is an integrated, India-statutory-first finance suite (a client-side SPA). The comparison below is about functional design, compliance depth and UX — areas where NEXA matches or beats far heavier products — not about backend scale or infrastructure, where tier-1 ERPs (SAP, NetSuite, Dynamics 365) remain the enterprise systems of record.</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1894,8 @@
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="46" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="46" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1958,7 +1959,12 @@
           <t xml:space="preserve">Oracle NetSuite</t>
         </is>
       </c>
-      <c r="J4" s="20" t="inlineStr">
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamics 365</t>
+        </is>
+      </c>
+      <c r="K4" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">NEXA edge</t>
         </is>
@@ -1979,6 +1985,7 @@
       <c r="H5" s="14"/>
       <c r="I5" s="14"/>
       <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -2026,7 +2033,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J6" s="22" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Baseline — NEXA matches all</t>
         </is>
@@ -2078,7 +2090,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J7" s="22" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K7" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Petty cash, reimb., P2P, IC, assets ALL post real vouchers</t>
         </is>
@@ -2130,7 +2147,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J8" s="22" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K8" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Standard everywhere</t>
         </is>
@@ -2182,7 +2204,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J9" s="22" t="inlineStr">
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K9" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Real contra/payment vouchers, not a memo ledger</t>
         </is>
@@ -2234,7 +2261,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Accrual on approve, payment on pay</t>
         </is>
@@ -2286,7 +2318,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J11" s="22" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K11" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Group + inter-company native</t>
         </is>
@@ -2307,6 +2344,7 @@
       <c r="H12" s="14"/>
       <c r="I12" s="14"/>
       <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -2354,7 +2392,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J13" s="22" t="inlineStr">
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K13" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Built-in vs localisation add-ons</t>
         </is>
@@ -2406,7 +2449,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K14" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Explicit UT detection + return folding</t>
         </is>
@@ -2458,7 +2506,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J15" s="22" t="inlineStr">
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K15" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Reconciling returns out-of-box</t>
         </is>
@@ -2510,7 +2563,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K16" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Invoice/rate/HSN-wise registers</t>
         </is>
@@ -2562,7 +2620,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J17" s="22" t="inlineStr">
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K17" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">LDC rate auto-applied</t>
         </is>
@@ -2614,7 +2677,12 @@
           <t xml:space="preserve">○  None</t>
         </is>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">○  None</t>
+        </is>
+      </c>
+      <c r="K18" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Newest rule — most rivals lack it</t>
         </is>
@@ -2666,7 +2734,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J19" s="22" t="inlineStr">
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K19" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Statutory schedules native</t>
         </is>
@@ -2687,6 +2760,7 @@
       <c r="H20" s="14"/>
       <c r="I20" s="14"/>
       <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -2734,7 +2808,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J21" s="22" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K21" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Tied to GL gross block</t>
         </is>
@@ -2786,7 +2865,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J22" s="22" t="inlineStr">
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K22" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Posts the book charge to GL</t>
         </is>
@@ -2838,7 +2922,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J23" s="22" t="inlineStr">
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K23" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Tax book alongside the book book</t>
         </is>
@@ -2890,7 +2979,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J24" s="22" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K24" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Procurement → asset with no rekey</t>
         </is>
@@ -2911,6 +3005,7 @@
       <c r="H25" s="14"/>
       <c r="I25" s="14"/>
       <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -2958,7 +3053,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J26" s="22" t="inlineStr">
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K26" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
@@ -3010,7 +3110,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J27" s="22" t="inlineStr">
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K27" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Enterprise control in a light app</t>
         </is>
@@ -3062,7 +3167,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J28" s="22" t="inlineStr">
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K28" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Accrual-accurate, tier-1 pattern</t>
         </is>
@@ -3114,7 +3224,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J29" s="22" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K29" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Inventory/Opex/Capex/Employee buckets</t>
         </is>
@@ -3166,7 +3281,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J30" s="22" t="inlineStr">
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K30" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
@@ -3187,6 +3307,7 @@
       <c r="H31" s="14"/>
       <c r="I31" s="14"/>
       <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -3234,7 +3355,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J32" s="22" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K32" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">In-suite, not a separate purchase</t>
         </is>
@@ -3286,7 +3412,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J33" s="22" t="inlineStr">
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K33" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
@@ -3338,7 +3469,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J34" s="22" t="inlineStr">
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K34" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
@@ -3390,7 +3526,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J35" s="22" t="inlineStr">
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K35" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Linked to P2P + GL</t>
         </is>
@@ -3411,6 +3552,7 @@
       <c r="H36" s="14"/>
       <c r="I36" s="14"/>
       <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -3458,7 +3600,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J37" s="22" t="inlineStr">
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K37" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
@@ -3510,7 +3657,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J38" s="22" t="inlineStr">
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K38" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Sale in A = purchase in B automatically</t>
         </is>
@@ -3562,7 +3714,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J39" s="22" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K39" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Group reporting native</t>
         </is>
@@ -3583,6 +3740,7 @@
       <c r="H40" s="14"/>
       <c r="I40" s="14"/>
       <c r="J40" s="14"/>
+      <c r="K40" s="14"/>
     </row>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
@@ -3630,7 +3788,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J41" s="22" t="inlineStr">
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K41" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Services P&amp;L</t>
         </is>
@@ -3682,7 +3845,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J42" s="22" t="inlineStr">
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K42" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Billable time</t>
         </is>
@@ -3734,7 +3902,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J43" s="22" t="inlineStr">
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K43" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Plan vs actual</t>
         </is>
@@ -3786,7 +3959,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J44" s="22" t="inlineStr">
+      <c r="J44" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K44" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Almost unique at this tier</t>
         </is>
@@ -3838,7 +4016,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J45" s="22" t="inlineStr">
+      <c r="J45" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">○  None</t>
+        </is>
+      </c>
+      <c r="K45" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Strategy in-suite</t>
         </is>
@@ -3890,7 +4073,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J46" s="22" t="inlineStr">
+      <c r="J46" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K46" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Statutory cost lens</t>
         </is>
@@ -3942,7 +4130,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J47" s="22" t="inlineStr">
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K47" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Shared filters across heads</t>
         </is>
@@ -3963,6 +4156,7 @@
       <c r="H48" s="14"/>
       <c r="I48" s="14"/>
       <c r="J48" s="14"/>
+      <c r="K48" s="14"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
@@ -4010,7 +4204,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J49" s="22" t="inlineStr">
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K49" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">In-suite pay run</t>
         </is>
@@ -4062,7 +4261,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J50" s="22" t="inlineStr">
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K50" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Workforce admin</t>
         </is>
@@ -4114,7 +4318,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J51" s="22" t="inlineStr">
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K51" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Hiring in the same suite</t>
         </is>
@@ -4166,7 +4375,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J52" s="22" t="inlineStr">
+      <c r="J52" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">○  None</t>
+        </is>
+      </c>
+      <c r="K52" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Rare even in big ERP</t>
         </is>
@@ -4218,7 +4432,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J53" s="22" t="inlineStr">
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K53" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">With global approvals bell</t>
         </is>
@@ -4239,6 +4458,7 @@
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
       <c r="J54" s="14"/>
+      <c r="K54" s="14"/>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
@@ -4286,7 +4506,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J55" s="22" t="inlineStr">
+      <c r="J55" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">○  None</t>
+        </is>
+      </c>
+      <c r="K55" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Keyboard-first nav, per-user shortcuts</t>
         </is>
@@ -4338,7 +4563,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J56" s="22" t="inlineStr">
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K56" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Auto-suggests reconciliation matches</t>
         </is>
@@ -4390,7 +4620,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J57" s="22" t="inlineStr">
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K57" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">postMany bulk posting path</t>
         </is>
@@ -4442,7 +4677,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J58" s="22" t="inlineStr">
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K58" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">jsPDF, dynamically imported</t>
         </is>
@@ -4494,7 +4734,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J59" s="22" t="inlineStr">
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K59" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Idempotent, deterministic narration</t>
         </is>
@@ -4546,7 +4791,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J60" s="22" t="inlineStr">
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K60" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Touchless AP within 2% tolerance</t>
         </is>
@@ -4598,7 +4848,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J61" s="22" t="inlineStr">
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K61" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Preparer ≠ approver enforced</t>
         </is>
@@ -4619,6 +4874,7 @@
       <c r="H62" s="14"/>
       <c r="I62" s="14"/>
       <c r="J62" s="14"/>
+      <c r="K62" s="14"/>
     </row>
     <row r="63">
       <c r="A63" s="16" t="inlineStr">
@@ -4666,7 +4922,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J63" s="22" t="inlineStr">
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K63" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Admin sees exactly what a user sees</t>
         </is>
@@ -4718,7 +4979,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J64" s="22" t="inlineStr">
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K64" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Turn functions on/off per tenant</t>
         </is>
@@ -4770,7 +5036,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J65" s="22" t="inlineStr">
+      <c r="J65" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">◐  Partial</t>
+        </is>
+      </c>
+      <c r="K65" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Workbooks recompute on open</t>
         </is>
@@ -4822,7 +5093,12 @@
           <t xml:space="preserve">●  Native</t>
         </is>
       </c>
-      <c r="J66" s="22" t="inlineStr">
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K66" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Browser-native</t>
         </is>
@@ -4874,7 +5150,12 @@
           <t xml:space="preserve">◐  Partial</t>
         </is>
       </c>
-      <c r="J67" s="22" t="inlineStr">
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">●  Native</t>
+        </is>
+      </c>
+      <c r="K67" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Familiar &amp; fast</t>
         </is>
@@ -4926,7 +5207,12 @@
           <t xml:space="preserve">○  None</t>
         </is>
       </c>
-      <c r="J68" s="22" t="inlineStr">
+      <c r="J68" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">○  None</t>
+        </is>
+      </c>
+      <c r="K68" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Instant vs months of rollout</t>
         </is>
@@ -4934,8 +5220,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -4994,7 +5280,7 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Matches Tally/Zoho on Indian statutory and goes further (MSME 43B(h), sec.197 LDC) — while bundling full ERP breadth those tools don't have. SAP/NetSuite need paid localisation; QuickBooks dropped India entirely.</t>
+          <t xml:space="preserve">Matches Tally/Zoho on Indian statutory and goes further (MSME 43B(h), sec.197 LDC) — while bundling full ERP breadth those tools don't have. SAP/NetSuite/Dynamics 365 need paid localisation; QuickBooks dropped India entirely.</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5314,7 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">These are the controls you normally only get after a six-figure SAP/NetSuite implementation — here with zero setup.</t>
+          <t xml:space="preserve">These are the controls you normally only get after a six-figure SAP/NetSuite/Dynamics implementation — here with zero setup.</t>
         </is>
       </c>
     </row>
@@ -5062,7 +5348,7 @@
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capex appraisal and business planning are essentially absent from Tally/Zoho/QuickBooks and are add-ons even in SAP/NetSuite.</t>
+          <t xml:space="preserve">Capex appraisal and business planning are essentially absent from Tally/Zoho/QuickBooks and are add-ons even in SAP/NetSuite/Dynamics 365.</t>
         </is>
       </c>
     </row>
@@ -5147,7 +5433,7 @@
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zoho needs Books+CRM+People+Recruit+Expense+Projects as separate apps; QuickBooks needs add-ons; NEXA is unified.</t>
+          <t xml:space="preserve">Zoho needs Books+CRM+People+Recruit+Expense+Projects as separate apps; Dynamics 365 spreads across Finance, BC, Sales, HR and Project Operations modules; QuickBooks needs add-ons. NEXA is unified.</t>
         </is>
       </c>
     </row>
@@ -5164,7 +5450,7 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP/NetSuite are large implementation projects; Tally is desktop-bound. NEXA runs in a browser immediately.</t>
+          <t xml:space="preserve">SAP/NetSuite/Dynamics 365 are large implementation projects costing months and significant professional-services fees; Tally is desktop-bound. NEXA runs in a browser immediately.</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5463,7 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">NEXA is a client-side SPA (browser localStorage), so it is not yet a multi-user, server-backed system of record at SAP/NetSuite scale. Its edge is functional design, India-compliance depth and UX — not infrastructure or enterprise data volume.</t>
+          <t xml:space="preserve">NEXA is a client-side SPA (browser localStorage), so it is not yet a multi-user, server-backed system of record at SAP/NetSuite/Dynamics scale. Its edge is functional design, India-compliance depth and UX — not infrastructure or enterprise data volume.</t>
         </is>
       </c>
       <c r="C17" s="26"/>
@@ -5524,6 +5810,7 @@
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -5587,6 +5874,11 @@
           <t xml:space="preserve">Oracle NetSuite</t>
         </is>
       </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamics 365</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
@@ -5618,6 +5910,9 @@
       <c r="I5" s="27">
         <v>1</v>
       </c>
+      <c r="J5" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
@@ -5649,6 +5944,9 @@
       <c r="I6" s="27">
         <v>1</v>
       </c>
+      <c r="J6" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
@@ -5680,6 +5978,9 @@
       <c r="I7" s="27">
         <v>1</v>
       </c>
+      <c r="J7" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
@@ -5711,6 +6012,9 @@
       <c r="I8" s="28">
         <v>0.5</v>
       </c>
+      <c r="J8" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
@@ -5742,6 +6046,9 @@
       <c r="I9" s="27">
         <v>1</v>
       </c>
+      <c r="J9" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
@@ -5773,6 +6080,9 @@
       <c r="I10" s="27">
         <v>1</v>
       </c>
+      <c r="J10" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
@@ -5804,6 +6114,9 @@
       <c r="I11" s="28">
         <v>0.5</v>
       </c>
+      <c r="J11" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
@@ -5835,6 +6148,9 @@
       <c r="I12" s="28">
         <v>0.5</v>
       </c>
+      <c r="J12" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
@@ -5866,6 +6182,9 @@
       <c r="I13" s="28">
         <v>0.5</v>
       </c>
+      <c r="J13" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
@@ -5897,6 +6216,9 @@
       <c r="I14" s="28">
         <v>0.5</v>
       </c>
+      <c r="J14" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
@@ -5928,6 +6250,9 @@
       <c r="I15" s="28">
         <v>0.5</v>
       </c>
+      <c r="J15" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
@@ -5959,6 +6284,9 @@
       <c r="I16" s="29">
         <v>0</v>
       </c>
+      <c r="J16" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -5990,6 +6318,9 @@
       <c r="I17" s="28">
         <v>0.5</v>
       </c>
+      <c r="J17" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -6021,6 +6352,9 @@
       <c r="I18" s="27">
         <v>1</v>
       </c>
+      <c r="J18" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
@@ -6052,6 +6386,9 @@
       <c r="I19" s="28">
         <v>0.5</v>
       </c>
+      <c r="J19" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
@@ -6083,6 +6420,9 @@
       <c r="I20" s="28">
         <v>0.5</v>
       </c>
+      <c r="J20" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
@@ -6114,6 +6454,9 @@
       <c r="I21" s="28">
         <v>0.5</v>
       </c>
+      <c r="J21" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="17" t="inlineStr">
@@ -6145,6 +6488,9 @@
       <c r="I22" s="27">
         <v>1</v>
       </c>
+      <c r="J22" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
@@ -6176,6 +6522,9 @@
       <c r="I23" s="27">
         <v>1</v>
       </c>
+      <c r="J23" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
@@ -6207,6 +6556,9 @@
       <c r="I24" s="27">
         <v>1</v>
       </c>
+      <c r="J24" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
@@ -6238,6 +6590,9 @@
       <c r="I25" s="28">
         <v>0.5</v>
       </c>
+      <c r="J25" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
@@ -6269,6 +6624,9 @@
       <c r="I26" s="27">
         <v>1</v>
       </c>
+      <c r="J26" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
@@ -6300,6 +6658,9 @@
       <c r="I27" s="27">
         <v>1</v>
       </c>
+      <c r="J27" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
@@ -6331,6 +6692,9 @@
       <c r="I28" s="27">
         <v>1</v>
       </c>
+      <c r="J28" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
@@ -6362,6 +6726,9 @@
       <c r="I29" s="27">
         <v>1</v>
       </c>
+      <c r="J29" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
@@ -6393,6 +6760,9 @@
       <c r="I30" s="27">
         <v>1</v>
       </c>
+      <c r="J30" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
@@ -6424,6 +6794,9 @@
       <c r="I31" s="27">
         <v>1</v>
       </c>
+      <c r="J31" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
@@ -6455,6 +6828,9 @@
       <c r="I32" s="27">
         <v>1</v>
       </c>
+      <c r="J32" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
@@ -6486,6 +6862,9 @@
       <c r="I33" s="27">
         <v>1</v>
       </c>
+      <c r="J33" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
@@ -6517,6 +6896,9 @@
       <c r="I34" s="27">
         <v>1</v>
       </c>
+      <c r="J34" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
@@ -6548,6 +6930,9 @@
       <c r="I35" s="27">
         <v>1</v>
       </c>
+      <c r="J35" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
@@ -6579,6 +6964,9 @@
       <c r="I36" s="27">
         <v>1</v>
       </c>
+      <c r="J36" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
@@ -6610,6 +6998,9 @@
       <c r="I37" s="28">
         <v>0.5</v>
       </c>
+      <c r="J37" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
@@ -6641,6 +7032,9 @@
       <c r="I38" s="28">
         <v>0.5</v>
       </c>
+      <c r="J38" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="17" t="inlineStr">
@@ -6672,6 +7066,9 @@
       <c r="I39" s="27">
         <v>1</v>
       </c>
+      <c r="J39" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
@@ -6703,6 +7100,9 @@
       <c r="I40" s="27">
         <v>1</v>
       </c>
+      <c r="J40" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
@@ -6734,6 +7134,9 @@
       <c r="I41" s="28">
         <v>0.5</v>
       </c>
+      <c r="J41" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
@@ -6765,6 +7168,9 @@
       <c r="I42" s="28">
         <v>0.5</v>
       </c>
+      <c r="J42" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
@@ -6796,6 +7202,9 @@
       <c r="I43" s="28">
         <v>0.5</v>
       </c>
+      <c r="J43" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
@@ -6827,6 +7236,9 @@
       <c r="I44" s="28">
         <v>0.5</v>
       </c>
+      <c r="J44" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
@@ -6858,6 +7270,9 @@
       <c r="I45" s="27">
         <v>1</v>
       </c>
+      <c r="J45" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
@@ -6889,6 +7304,9 @@
       <c r="I46" s="27">
         <v>1</v>
       </c>
+      <c r="J46" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
@@ -6920,6 +7338,9 @@
       <c r="I47" s="27">
         <v>1</v>
       </c>
+      <c r="J47" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
@@ -6951,6 +7372,9 @@
       <c r="I48" s="27">
         <v>1</v>
       </c>
+      <c r="J48" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
@@ -6982,6 +7406,9 @@
       <c r="I49" s="27">
         <v>1</v>
       </c>
+      <c r="J49" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="17" t="inlineStr">
@@ -7013,6 +7440,9 @@
       <c r="I50" s="27">
         <v>1</v>
       </c>
+      <c r="J50" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
@@ -7044,6 +7474,9 @@
       <c r="I51" s="27">
         <v>1</v>
       </c>
+      <c r="J51" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="17" t="inlineStr">
@@ -7075,6 +7508,9 @@
       <c r="I52" s="27">
         <v>1</v>
       </c>
+      <c r="J52" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="17" t="inlineStr">
@@ -7106,6 +7542,9 @@
       <c r="I53" s="27">
         <v>1</v>
       </c>
+      <c r="J53" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="17" t="inlineStr">
@@ -7137,6 +7576,9 @@
       <c r="I54" s="27">
         <v>1</v>
       </c>
+      <c r="J54" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="17" t="inlineStr">
@@ -7168,6 +7610,9 @@
       <c r="I55" s="28">
         <v>0.5</v>
       </c>
+      <c r="J55" s="28">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="17" t="inlineStr">
@@ -7199,6 +7644,9 @@
       <c r="I56" s="27">
         <v>1</v>
       </c>
+      <c r="J56" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
@@ -7230,6 +7678,9 @@
       <c r="I57" s="28">
         <v>0.5</v>
       </c>
+      <c r="J57" s="27">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="17" t="inlineStr">
@@ -7261,6 +7712,9 @@
       <c r="I58" s="29">
         <v>0</v>
       </c>
+      <c r="J58" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="30" t="inlineStr">
@@ -7300,6 +7754,10 @@
         <f>SUM(I5:I58)</f>
         <v>0</v>
       </c>
+      <c r="J59" s="31">
+        <f>SUM(J5:J58)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="32" t="inlineStr">
@@ -7339,11 +7797,15 @@
         <f>I59/54</f>
         <v>0</v>
       </c>
+      <c r="J60" s="33">
+        <f>J59/54</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>